<commit_message>
updated validation and downloading error excel
</commit_message>
<xml_diff>
--- a/Backend/templates/CUSTOM_Fee_Upload_Template.xlsx
+++ b/Backend/templates/CUSTOM_Fee_Upload_Template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>htNumber</t>
   </si>
@@ -20,12 +20,6 @@
   </si>
   <si>
     <t>amount</t>
-  </si>
-  <si>
-    <t>paymentDate</t>
-  </si>
-  <si>
-    <t>academicYear</t>
   </si>
 </sst>
 </file>
@@ -402,10 +396,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -415,12 +409,6 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>